<commit_message>
Reports: July 2026 H1 (5 report(s))
</commit_message>
<xml_diff>
--- a/Payroll Report/archive/Payroll_Report_July_2026_H1.xlsx
+++ b/Payroll Report/archive/Payroll_Report_July_2026_H1.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="35">
   <si>
     <t>Employee</t>
   </si>
@@ -90,16 +90,10 @@
     <t>July 2026 H1  (2026-07-01 to 2026-07-14 inclusive)</t>
   </si>
   <si>
-    <t>Run date (UTC)</t>
-  </si>
-  <si>
-    <t>2026-07-16</t>
-  </si>
-  <si>
     <t>Generated (UTC)</t>
   </si>
   <si>
-    <t>2026-07-16 07:14:31</t>
+    <t>2026-07-16 09:59:51</t>
   </si>
   <si>
     <t>Source</t>
@@ -409,7 +403,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="18.484375" customWidth="true" bestFit="true"/>
@@ -472,14 +466,6 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="B8" t="s" s="0">
-        <v>36</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>